<commit_message>
Update July OHIGGINS Metrogas invoice
Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/OHIGGINS/Gastos_OHIGGINS_2026.xlsx
+++ b/OHIGGINS/Gastos_OHIGGINS_2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Detalle" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1" forceFullCalc="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -160,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +181,8 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -697,6 +699,10 @@
       <c r="I5" t="n">
         <v>829490</v>
       </c>
+      <c r="P5">
+        <f>SUM(D5:O5)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -737,7 +743,7 @@
       <c r="N6" s="5" t="n"/>
       <c r="O6" s="5" t="n"/>
       <c r="P6" s="5">
-        <f>SUM(D5:O5)</f>
+        <f>SUM(D6:O6)</f>
         <v/>
       </c>
     </row>
@@ -778,7 +784,7 @@
       <c r="N7" s="5" t="n"/>
       <c r="O7" s="5" t="n"/>
       <c r="P7" s="5">
-        <f>SUM(D6:O6)</f>
+        <f>SUM(D7:O7)</f>
         <v/>
       </c>
     </row>
@@ -821,7 +827,7 @@
       <c r="N8" s="5" t="n"/>
       <c r="O8" s="5" t="n"/>
       <c r="P8" s="5">
-        <f>SUM(D7:O7)</f>
+        <f>SUM(D8:O8)</f>
         <v/>
       </c>
     </row>
@@ -854,7 +860,7 @@
         <v>4984</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>5208</v>
+        <v>5209</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="5" t="n"/>
@@ -862,7 +868,7 @@
       <c r="N9" s="5" t="n"/>
       <c r="O9" s="5" t="n"/>
       <c r="P9" s="5">
-        <f>SUM(D8:O8)</f>
+        <f>SUM(D9:O9)</f>
         <v/>
       </c>
     </row>
@@ -883,7 +889,7 @@
       <c r="N10" s="5" t="n"/>
       <c r="O10" s="5" t="n"/>
       <c r="P10" s="5">
-        <f>SUM(D9:O9)</f>
+        <f>SUM(D10:O10)</f>
         <v/>
       </c>
     </row>
@@ -904,7 +910,7 @@
       <c r="N11" s="5" t="n"/>
       <c r="O11" s="5" t="n"/>
       <c r="P11" s="5">
-        <f>SUM(D10:O10)</f>
+        <f>SUM(D11:O11)</f>
         <v/>
       </c>
     </row>
@@ -925,7 +931,7 @@
       <c r="N12" s="5" t="n"/>
       <c r="O12" s="5" t="n"/>
       <c r="P12" s="5">
-        <f>SUM(D11:O11)</f>
+        <f>SUM(D12:O12)</f>
         <v/>
       </c>
     </row>
@@ -946,7 +952,7 @@
       <c r="N13" s="5" t="n"/>
       <c r="O13" s="5" t="n"/>
       <c r="P13" s="5">
-        <f>SUM(D12:O12)</f>
+        <f>SUM(D13:O13)</f>
         <v/>
       </c>
     </row>
@@ -967,7 +973,7 @@
       <c r="N14" s="5" t="n"/>
       <c r="O14" s="5" t="n"/>
       <c r="P14" s="5">
-        <f>SUM(D13:O13)</f>
+        <f>SUM(D14:O14)</f>
         <v/>
       </c>
     </row>
@@ -988,7 +994,7 @@
       <c r="N15" s="5" t="n"/>
       <c r="O15" s="5" t="n"/>
       <c r="P15" s="5">
-        <f>SUM(D14:O14)</f>
+        <f>SUM(D15:O15)</f>
         <v/>
       </c>
     </row>
@@ -1009,7 +1015,7 @@
       <c r="N16" s="5" t="n"/>
       <c r="O16" s="5" t="n"/>
       <c r="P16" s="5">
-        <f>SUM(D15:O15)</f>
+        <f>SUM(D16:O16)</f>
         <v/>
       </c>
     </row>
@@ -1030,7 +1036,7 @@
       <c r="N17" s="5" t="n"/>
       <c r="O17" s="5" t="n"/>
       <c r="P17" s="5">
-        <f>SUM(D16:O16)</f>
+        <f>SUM(D17:O17)</f>
         <v/>
       </c>
     </row>
@@ -1051,7 +1057,7 @@
       <c r="N18" s="5" t="n"/>
       <c r="O18" s="5" t="n"/>
       <c r="P18" s="5">
-        <f>SUM(D17:O17)</f>
+        <f>SUM(D18:O18)</f>
         <v/>
       </c>
     </row>
@@ -1072,7 +1078,7 @@
       <c r="N19" s="5" t="n"/>
       <c r="O19" s="5" t="n"/>
       <c r="P19" s="5">
-        <f>SUM(D18:O18)</f>
+        <f>SUM(D19:O19)</f>
         <v/>
       </c>
     </row>
@@ -1093,7 +1099,7 @@
       <c r="N20" s="5" t="n"/>
       <c r="O20" s="5" t="n"/>
       <c r="P20" s="5">
-        <f>SUM(D19:O19)</f>
+        <f>SUM(D20:O20)</f>
         <v/>
       </c>
     </row>
@@ -1106,55 +1112,55 @@
       <c r="B21" s="11" t="n"/>
       <c r="C21" s="12" t="n"/>
       <c r="D21" s="7">
-        <f>SUM(D5:D19)</f>
+        <f>SUM(D5:D20)</f>
         <v/>
       </c>
       <c r="E21" s="7">
-        <f>SUM(E5:E19)</f>
+        <f>SUM(E5:E20)</f>
         <v/>
       </c>
       <c r="F21" s="7">
-        <f>SUM(F5:F19)</f>
+        <f>SUM(F5:F20)</f>
         <v/>
       </c>
       <c r="G21" s="7">
-        <f>SUM(G5:G19)</f>
+        <f>SUM(G5:G20)</f>
         <v/>
       </c>
       <c r="H21" s="7">
-        <f>SUM(H5:H19)</f>
+        <f>SUM(H5:H20)</f>
         <v/>
       </c>
       <c r="I21" s="7">
-        <f>SUM(I5:I19)</f>
+        <f>SUM(I5:I20)</f>
         <v/>
       </c>
       <c r="J21" s="7">
-        <f>SUM(J5:J19)</f>
+        <f>SUM(J5:J20)</f>
         <v/>
       </c>
       <c r="K21" s="7">
-        <f>SUM(K5:K19)</f>
+        <f>SUM(K5:K20)</f>
         <v/>
       </c>
       <c r="L21" s="7">
-        <f>SUM(L5:L19)</f>
+        <f>SUM(L5:L20)</f>
         <v/>
       </c>
       <c r="M21" s="7">
-        <f>SUM(M5:M19)</f>
+        <f>SUM(M5:M20)</f>
         <v/>
       </c>
       <c r="N21" s="7">
-        <f>SUM(N5:N19)</f>
+        <f>SUM(N5:N20)</f>
         <v/>
       </c>
       <c r="O21" s="7">
-        <f>SUM(O5:O19)</f>
+        <f>SUM(O5:O20)</f>
         <v/>
       </c>
       <c r="P21" s="7">
-        <f>SUM(P5:P19)</f>
+        <f>SUM(P5:P20)</f>
         <v/>
       </c>
     </row>
@@ -1625,8 +1631,8 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n">
-        <v>46209</v>
+      <c r="A16" s="18" t="n">
+        <v>46233</v>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
@@ -1640,20 +1646,20 @@
       </c>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>Metrogas — INVALMAR SRL · O'Higgins 2225</t>
-        </is>
-      </c>
-      <c r="E16" s="17" t="n">
-        <v>5208</v>
+          <t>Metrogas — INVALMAR SRL · O'Higgins 2225 · período 02/06/2026 a 01/07/2026</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>5209</v>
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>Mercado Pago / Gmail</t>
+          <t>Factura Metrogas · Débito automático NO</t>
         </is>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>10139236800</t>
+          <t>Cliente 10139236800 · medidor 8683287 · lectura real · original $5.208,73</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix OHIGGINS Metrogas months by bill period; add July pending.
Reassign paid MP Metrogas entries one month earlier (pago jul→junio),
and load July bill $5208.73 (ceil $5209) due 14-ago as unpaid.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/OHIGGINS/Gastos_OHIGGINS_2026.xlsx
+++ b/OHIGGINS/Gastos_OHIGGINS_2026.xlsx
@@ -577,7 +577,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>OHIGGINS · ABL 3016365 · Edenor Chagas 9267222037 · Metrogas INVALMAR 10139236800 · Personal TV · Expensas 2219 piso 8 (Copropi/Kalmus)</t>
+          <t>OHIGGINS · ABL 3016365 · Edenor Chagas 9267222037 · Metrogas INVALMAR 10139236800 (mes=período boleta) · Personal TV · Expensas 2219 piso 8 (Copropi/Kalmus)</t>
         </is>
       </c>
     </row>
@@ -843,18 +843,20 @@
       </c>
       <c r="D9" s="5" t="n"/>
       <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
+      <c r="F9" s="5" t="n">
+        <v>4850</v>
+      </c>
       <c r="G9" s="5" t="n">
-        <v>4850</v>
+        <v>4935</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>4935</v>
+        <v>4984</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>4984</v>
+        <v>5208</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>5208</v>
+        <v>5209</v>
       </c>
       <c r="K9" s="5" t="n"/>
       <c r="L9" s="5" t="n"/>
@@ -1172,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1541,7 +1543,7 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>Metrogas — INVALMAR SRL · O'Higgins 2225</t>
+          <t>Metrogas — INVALMAR SRL · O'Higgins 2225 · marzo (pago 6-abr)</t>
         </is>
       </c>
       <c r="E13" s="17" t="n">
@@ -1554,13 +1556,13 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>10139236800</t>
+          <t>10139236800 · período marzo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="n">
-        <v>46146</v>
+        <v>46150</v>
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
@@ -1574,7 +1576,7 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>Metrogas — INVALMAR SRL · O'Higgins 2225</t>
+          <t>Metrogas — INVALMAR SRL · O'Higgins 2225 · abril (pago 8-may)</t>
         </is>
       </c>
       <c r="E14" s="17" t="n">
@@ -1587,13 +1589,13 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>10139236800</t>
+          <t>10139236800 · período abril</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="n">
-        <v>46175</v>
+        <v>46176</v>
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
@@ -1607,7 +1609,7 @@
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>Metrogas — INVALMAR SRL · O'Higgins 2225</t>
+          <t>Metrogas — INVALMAR SRL · O'Higgins 2225 · mayo (pago 3-jun)</t>
         </is>
       </c>
       <c r="E15" s="17" t="n">
@@ -1620,13 +1622,13 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>10139236800</t>
+          <t>10139236800 · período mayo</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="16" t="n">
-        <v>46209</v>
+        <v>46217</v>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
@@ -1640,7 +1642,7 @@
       </c>
       <c r="D16" s="17" t="inlineStr">
         <is>
-          <t>Metrogas — INVALMAR SRL · O'Higgins 2225</t>
+          <t>Metrogas — INVALMAR SRL · O'Higgins 2225 · junio (pago 14-jul)</t>
         </is>
       </c>
       <c r="E16" s="17" t="n">
@@ -1653,13 +1655,13 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>10139236800</t>
+          <t>10139236800 · período junio</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="n">
-        <v>46032</v>
+        <v>46248</v>
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
@@ -1668,31 +1670,31 @@
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>TV CABLE-INTERNET</t>
+          <t>GAS</t>
         </is>
       </c>
       <c r="D17" s="17" t="inlineStr">
         <is>
-          <t>Personal — Pago directo</t>
+          <t>Metrogas — INVALMAR SRL · O'Higgins 2225 · julio (vence 14-ago · pendiente)</t>
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>34921</v>
+        <v>5209</v>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>Mercado Pago</t>
+          <t>Pendiente · vence 14-ago-2026</t>
         </is>
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>Personal flow · resumen MP</t>
+          <t>10139236800 · período julio · factura $5208.73</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="16" t="n">
-        <v>46122</v>
+        <v>46032</v>
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
@@ -1710,7 +1712,7 @@
         </is>
       </c>
       <c r="E18" s="17" t="n">
-        <v>101114</v>
+        <v>34921</v>
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
@@ -1719,13 +1721,13 @@
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
-          <t>resumen MP</t>
+          <t>Personal flow · resumen MP</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="n">
-        <v>46154</v>
+        <v>46122</v>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
@@ -1743,7 +1745,7 @@
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>53245</v>
+        <v>101114</v>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
@@ -1758,7 +1760,7 @@
     </row>
     <row r="20">
       <c r="A20" s="16" t="n">
-        <v>46184</v>
+        <v>46154</v>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
@@ -1776,7 +1778,7 @@
         </is>
       </c>
       <c r="E20" s="17" t="n">
-        <v>55106</v>
+        <v>53245</v>
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
@@ -1791,7 +1793,7 @@
     </row>
     <row r="21">
       <c r="A21" s="16" t="n">
-        <v>46217</v>
+        <v>46184</v>
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
@@ -1809,7 +1811,7 @@
         </is>
       </c>
       <c r="E21" s="17" t="n">
-        <v>56200</v>
+        <v>55106</v>
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
@@ -1824,7 +1826,7 @@
     </row>
     <row r="22">
       <c r="A22" s="16" t="n">
-        <v>46031</v>
+        <v>46217</v>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
@@ -1833,31 +1835,31 @@
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>EXPENSAS</t>
+          <t>TV CABLE-INTERNET</t>
         </is>
       </c>
       <c r="D22" s="17" t="inlineStr">
         <is>
-          <t>Expensas OHIGGINS 2219 piso 8 · enero</t>
+          <t>Personal — Pago directo</t>
         </is>
       </c>
       <c r="E22" s="17" t="n">
-        <v>376564</v>
+        <v>56200</v>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>Mercado Pago — Consorcio De Copropi</t>
+          <t>Mercado Pago</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr">
         <is>
-          <t>Kalmus</t>
+          <t>resumen MP</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="n">
-        <v>46059</v>
+        <v>46031</v>
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
@@ -1871,11 +1873,11 @@
       </c>
       <c r="D23" s="17" t="inlineStr">
         <is>
-          <t>Expensas OHIGGINS 2219 piso 8 · febrero</t>
+          <t>Expensas OHIGGINS 2219 piso 8 · enero</t>
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>395551</v>
+        <v>376564</v>
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
@@ -1890,7 +1892,7 @@
     </row>
     <row r="24">
       <c r="A24" s="16" t="n">
-        <v>46091</v>
+        <v>46059</v>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
@@ -1904,11 +1906,11 @@
       </c>
       <c r="D24" s="17" t="inlineStr">
         <is>
-          <t>Expensas OHIGGINS 2219 piso 8 · marzo</t>
+          <t>Expensas OHIGGINS 2219 piso 8 · febrero</t>
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>402934</v>
+        <v>395551</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
@@ -1923,7 +1925,7 @@
     </row>
     <row r="25">
       <c r="A25" s="16" t="n">
-        <v>46120</v>
+        <v>46091</v>
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
@@ -1937,26 +1939,26 @@
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>Expensas OHIGGINS 2219 piso 8 · abril</t>
+          <t>Expensas OHIGGINS 2219 piso 8 · marzo</t>
         </is>
       </c>
       <c r="E25" s="17" t="n">
-        <v>570841</v>
+        <v>402934</v>
       </c>
       <c r="F25" s="17" t="inlineStr">
         <is>
-          <t>Banco — Transferencia</t>
+          <t>Mercado Pago — Consorcio De Copropi</t>
         </is>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>Gmail Sent 8-abr</t>
+          <t>Kalmus</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="16" t="n">
-        <v>46183</v>
+        <v>46120</v>
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
@@ -1970,51 +1972,84 @@
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t>Expensas OHIGGINS 2219 piso 8 · mayo (pago 10-jun)</t>
+          <t>Expensas OHIGGINS 2219 piso 8 · abril</t>
         </is>
       </c>
       <c r="E26" s="17" t="n">
-        <v>666347</v>
+        <v>570841</v>
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>Mercado Pago — Consorcio De Copropi</t>
+          <t>Banco — Transferencia</t>
         </is>
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>Gmail Sent</t>
+          <t>Gmail Sent 8-abr</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="16" t="n">
+        <v>46183</v>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>EXPENSAS</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>Expensas OHIGGINS 2219 piso 8 · mayo (pago 10-jun)</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="n">
+        <v>666347</v>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Mercado Pago — Consorcio De Copropi</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>Gmail Sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
         <v>46212</v>
       </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>SERVICIOS</t>
-        </is>
-      </c>
-      <c r="C27" s="17" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>SERVICIOS</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>EXPENSAS</t>
         </is>
       </c>
-      <c r="D27" s="17" t="inlineStr">
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>Expensas OHIGGINS 2219 piso 8 · junio (pago 9-jul)</t>
         </is>
       </c>
-      <c r="E27" s="17" t="n">
+      <c r="E28" s="17" t="n">
         <v>829490</v>
       </c>
-      <c r="F27" s="17" t="inlineStr">
+      <c r="F28" s="17" t="inlineStr">
         <is>
           <t>Mercado Pago — Consorcio De Copropi</t>
         </is>
       </c>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="G28" s="17" t="inlineStr">
         <is>
           <t>Gmail Sent</t>
         </is>

</xml_diff>

<commit_message>
Add OHIGGINS ABL August quota 08 (88891).
Register AGIP partida 3016365 with 1st due 14/08/2026; ceil from 88890.01.

Co-authored-by: solzito148 <solzito148@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/OHIGGINS/Gastos_OHIGGINS_2026.xlsx
+++ b/OHIGGINS/Gastos_OHIGGINS_2026.xlsx
@@ -160,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -181,6 +181,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -772,7 +773,9 @@
       <c r="J7" s="5" t="n">
         <v>88891</v>
       </c>
-      <c r="K7" s="5" t="n"/>
+      <c r="K7" s="5" t="n">
+        <v>88891</v>
+      </c>
       <c r="L7" s="5" t="n"/>
       <c r="M7" s="5" t="n"/>
       <c r="N7" s="5" t="n"/>
@@ -1172,7 +1175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2020,6 +2023,39 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="18" t="n">
+        <v>46248</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>IMPUESTOS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>ABL</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ABL — partida 3016365 · CUOTA 08/2026</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>88891</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Mercado Pago</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>3016365 · ceil desde $88.890,01 · 1° vto 14/08/2026 · 2° vto 31/08 $100.779</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>